<commit_message>
Master SKU sample: Margin, Auto Margin, Auto %, Manual Margin, Manual Settlement columns
</commit_message>
<xml_diff>
--- a/skuwisedata/master_sku_sample.xlsx
+++ b/skuwisedata/master_sku_sample.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X500"/>
+  <dimension ref="A1:AC500"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -464,9 +464,14 @@
     <col width="10" customWidth="1" min="19" max="19"/>
     <col width="8" customWidth="1" min="20" max="20"/>
     <col width="10" customWidth="1" min="21" max="21"/>
-    <col width="11" customWidth="1" min="22" max="22"/>
-    <col width="18" customWidth="1" min="23" max="23"/>
-    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="18" customWidth="1" min="26" max="26"/>
+    <col width="11" customWidth="1" min="27" max="27"/>
+    <col width="18" customWidth="1" min="28" max="28"/>
+    <col width="13" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -577,15 +582,40 @@
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
+          <t>Margin</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Auto Margin</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Auto %</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Manual Margin</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Manual Settlement</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
           <t>Final COP</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Expected Settlement</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Selling Price</t>
         </is>

</xml_diff>

<commit_message>
Master SKU sample: add Amazon Add Rs + Max Step % columns (31 cols)
</commit_message>
<xml_diff>
--- a/skuwisedata/master_sku_sample.xlsx
+++ b/skuwisedata/master_sku_sample.xlsx
@@ -1,46 +1,44 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20000" windowHeight="12000"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master SKU" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Master SKU" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
   <fonts count="2">
     <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <b/>
       <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F6FEB"/>
+        <fgColor rgb="FF1F6FEB"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -54,424 +52,74 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00E5E7EB"/>
+        <color rgb="FFE5E7EB"/>
       </left>
       <right style="thin">
-        <color rgb="00E5E7EB"/>
+        <color rgb="FFE5E7EB"/>
       </right>
       <top style="thin">
-        <color rgb="00E5E7EB"/>
+        <color rgb="FFE5E7EB"/>
       </top>
       <bottom style="thin">
-        <color rgb="00E5E7EB"/>
+        <color rgb="FFE5E7EB"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="1F497D"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="EEECE1"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="4F81BD"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="C0504D"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="9BBB59"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="8064A2"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="4BACC6"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="F79646"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0000FF"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="800080"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme name="Office">
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="35000">
-              <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="40000">
-              <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-</a:theme>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:AC500"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:AE500"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
-    <col width="20" customWidth="1" min="17" max="17"/>
-    <col width="10" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
-    <col width="8" customWidth="1" min="20" max="20"/>
-    <col width="10" customWidth="1" min="21" max="21"/>
-    <col width="14" customWidth="1" min="22" max="22"/>
-    <col width="14" customWidth="1" min="23" max="23"/>
-    <col width="14" customWidth="1" min="24" max="24"/>
-    <col width="14" customWidth="1" min="25" max="25"/>
-    <col width="18" customWidth="1" min="26" max="26"/>
-    <col width="11" customWidth="1" min="27" max="27"/>
-    <col width="18" customWidth="1" min="28" max="28"/>
-    <col width="13" customWidth="1" min="29" max="29"/>
+    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="11" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
+    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="8" max="8" width="13" customWidth="1"/>
+    <col min="9" max="9" width="11" customWidth="1"/>
+    <col min="10" max="10" width="14" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="12" max="12" width="22" customWidth="1"/>
+    <col min="13" max="13" width="10" customWidth="1"/>
+    <col min="14" max="14" width="14" customWidth="1"/>
+    <col min="15" max="15" width="18" customWidth="1"/>
+    <col min="16" max="16" width="20" customWidth="1"/>
+    <col min="17" max="17" width="20" customWidth="1"/>
+    <col min="18" max="18" width="10" customWidth="1"/>
+    <col min="19" max="19" width="10" customWidth="1"/>
+    <col min="20" max="20" width="8" customWidth="1"/>
+    <col min="21" max="21" width="10" customWidth="1"/>
+    <col min="22" max="22" width="14" customWidth="1"/>
+    <col min="23" max="23" width="14" customWidth="1"/>
+    <col min="24" max="24" width="14" customWidth="1"/>
+    <col min="25" max="25" width="14" customWidth="1"/>
+    <col min="26" max="26" width="18" customWidth="1"/>
+    <col min="27" max="27" width="14" customWidth="1"/>
+    <col min="28" max="28" width="12" customWidth="1"/>
+    <col min="29" max="29" width="11" customWidth="1"/>
+    <col min="30" max="30" width="18" customWidth="1"/>
+    <col min="31" max="31" width="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -607,3026 +255,2537 @@
       </c>
       <c r="AA1" s="1" t="inlineStr">
         <is>
+          <t>Amazon Add Rs</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>Max Step %</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
           <t>Final COP</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Expected Settlement</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Selling Price</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2">
+      <c r="A2" s="2">
         <f>IF(E2="","",COUNTA(E$2:E2))</f>
-        <v/>
       </c>
     </row>
     <row r="3">
-      <c r="A3">
+      <c r="A3" s="2">
         <f>IF(E3="","",COUNTA(E$2:E3))</f>
-        <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4">
+      <c r="A4" s="2">
         <f>IF(E4="","",COUNTA(E$2:E4))</f>
-        <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5">
+      <c r="A5" s="2">
         <f>IF(E5="","",COUNTA(E$2:E5))</f>
-        <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6">
+      <c r="A6" s="2">
         <f>IF(E6="","",COUNTA(E$2:E6))</f>
-        <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7">
+      <c r="A7" s="2">
         <f>IF(E7="","",COUNTA(E$2:E7))</f>
-        <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8">
+      <c r="A8" s="2">
         <f>IF(E8="","",COUNTA(E$2:E8))</f>
-        <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9">
+      <c r="A9" s="2">
         <f>IF(E9="","",COUNTA(E$2:E9))</f>
-        <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10">
+      <c r="A10" s="2">
         <f>IF(E10="","",COUNTA(E$2:E10))</f>
-        <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11">
+      <c r="A11" s="2">
         <f>IF(E11="","",COUNTA(E$2:E11))</f>
-        <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12">
+      <c r="A12" s="2">
         <f>IF(E12="","",COUNTA(E$2:E12))</f>
-        <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13">
+      <c r="A13" s="2">
         <f>IF(E13="","",COUNTA(E$2:E13))</f>
-        <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14">
+      <c r="A14" s="2">
         <f>IF(E14="","",COUNTA(E$2:E14))</f>
-        <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15">
+      <c r="A15" s="2">
         <f>IF(E15="","",COUNTA(E$2:E15))</f>
-        <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16">
+      <c r="A16" s="2">
         <f>IF(E16="","",COUNTA(E$2:E16))</f>
-        <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17">
+      <c r="A17" s="2">
         <f>IF(E17="","",COUNTA(E$2:E17))</f>
-        <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18">
+      <c r="A18" s="2">
         <f>IF(E18="","",COUNTA(E$2:E18))</f>
-        <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19">
+      <c r="A19" s="2">
         <f>IF(E19="","",COUNTA(E$2:E19))</f>
-        <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20">
+      <c r="A20" s="2">
         <f>IF(E20="","",COUNTA(E$2:E20))</f>
-        <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21">
+      <c r="A21" s="2">
         <f>IF(E21="","",COUNTA(E$2:E21))</f>
-        <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22">
+      <c r="A22" s="2">
         <f>IF(E22="","",COUNTA(E$2:E22))</f>
-        <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23">
+      <c r="A23" s="2">
         <f>IF(E23="","",COUNTA(E$2:E23))</f>
-        <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24">
+      <c r="A24" s="2">
         <f>IF(E24="","",COUNTA(E$2:E24))</f>
-        <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25">
+      <c r="A25" s="2">
         <f>IF(E25="","",COUNTA(E$2:E25))</f>
-        <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26">
+      <c r="A26" s="2">
         <f>IF(E26="","",COUNTA(E$2:E26))</f>
-        <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27">
+      <c r="A27" s="2">
         <f>IF(E27="","",COUNTA(E$2:E27))</f>
-        <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28">
+      <c r="A28" s="2">
         <f>IF(E28="","",COUNTA(E$2:E28))</f>
-        <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29">
+      <c r="A29" s="2">
         <f>IF(E29="","",COUNTA(E$2:E29))</f>
-        <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30">
+      <c r="A30" s="2">
         <f>IF(E30="","",COUNTA(E$2:E30))</f>
-        <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31">
+      <c r="A31" s="2">
         <f>IF(E31="","",COUNTA(E$2:E31))</f>
-        <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32">
+      <c r="A32" s="2">
         <f>IF(E32="","",COUNTA(E$2:E32))</f>
-        <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33">
+      <c r="A33" s="2">
         <f>IF(E33="","",COUNTA(E$2:E33))</f>
-        <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34">
+      <c r="A34" s="2">
         <f>IF(E34="","",COUNTA(E$2:E34))</f>
-        <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35">
+      <c r="A35" s="2">
         <f>IF(E35="","",COUNTA(E$2:E35))</f>
-        <v/>
       </c>
     </row>
     <row r="36">
-      <c r="A36">
+      <c r="A36" s="2">
         <f>IF(E36="","",COUNTA(E$2:E36))</f>
-        <v/>
       </c>
     </row>
     <row r="37">
-      <c r="A37">
+      <c r="A37" s="2">
         <f>IF(E37="","",COUNTA(E$2:E37))</f>
-        <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38">
+      <c r="A38" s="2">
         <f>IF(E38="","",COUNTA(E$2:E38))</f>
-        <v/>
       </c>
     </row>
     <row r="39">
-      <c r="A39">
+      <c r="A39" s="2">
         <f>IF(E39="","",COUNTA(E$2:E39))</f>
-        <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40">
+      <c r="A40" s="2">
         <f>IF(E40="","",COUNTA(E$2:E40))</f>
-        <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41">
+      <c r="A41" s="2">
         <f>IF(E41="","",COUNTA(E$2:E41))</f>
-        <v/>
       </c>
     </row>
     <row r="42">
-      <c r="A42">
+      <c r="A42" s="2">
         <f>IF(E42="","",COUNTA(E$2:E42))</f>
-        <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43">
+      <c r="A43" s="2">
         <f>IF(E43="","",COUNTA(E$2:E43))</f>
-        <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44">
+      <c r="A44" s="2">
         <f>IF(E44="","",COUNTA(E$2:E44))</f>
-        <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45">
+      <c r="A45" s="2">
         <f>IF(E45="","",COUNTA(E$2:E45))</f>
-        <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46">
+      <c r="A46" s="2">
         <f>IF(E46="","",COUNTA(E$2:E46))</f>
-        <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47">
+      <c r="A47" s="2">
         <f>IF(E47="","",COUNTA(E$2:E47))</f>
-        <v/>
       </c>
     </row>
     <row r="48">
-      <c r="A48">
+      <c r="A48" s="2">
         <f>IF(E48="","",COUNTA(E$2:E48))</f>
-        <v/>
       </c>
     </row>
     <row r="49">
-      <c r="A49">
+      <c r="A49" s="2">
         <f>IF(E49="","",COUNTA(E$2:E49))</f>
-        <v/>
       </c>
     </row>
     <row r="50">
-      <c r="A50">
+      <c r="A50" s="2">
         <f>IF(E50="","",COUNTA(E$2:E50))</f>
-        <v/>
       </c>
     </row>
     <row r="51">
-      <c r="A51">
+      <c r="A51" s="2">
         <f>IF(E51="","",COUNTA(E$2:E51))</f>
-        <v/>
       </c>
     </row>
     <row r="52">
-      <c r="A52">
+      <c r="A52" s="2">
         <f>IF(E52="","",COUNTA(E$2:E52))</f>
-        <v/>
       </c>
     </row>
     <row r="53">
-      <c r="A53">
+      <c r="A53" s="2">
         <f>IF(E53="","",COUNTA(E$2:E53))</f>
-        <v/>
       </c>
     </row>
     <row r="54">
-      <c r="A54">
+      <c r="A54" s="2">
         <f>IF(E54="","",COUNTA(E$2:E54))</f>
-        <v/>
       </c>
     </row>
     <row r="55">
-      <c r="A55">
+      <c r="A55" s="2">
         <f>IF(E55="","",COUNTA(E$2:E55))</f>
-        <v/>
       </c>
     </row>
     <row r="56">
-      <c r="A56">
+      <c r="A56" s="2">
         <f>IF(E56="","",COUNTA(E$2:E56))</f>
-        <v/>
       </c>
     </row>
     <row r="57">
-      <c r="A57">
+      <c r="A57" s="2">
         <f>IF(E57="","",COUNTA(E$2:E57))</f>
-        <v/>
       </c>
     </row>
     <row r="58">
-      <c r="A58">
+      <c r="A58" s="2">
         <f>IF(E58="","",COUNTA(E$2:E58))</f>
-        <v/>
       </c>
     </row>
     <row r="59">
-      <c r="A59">
+      <c r="A59" s="2">
         <f>IF(E59="","",COUNTA(E$2:E59))</f>
-        <v/>
       </c>
     </row>
     <row r="60">
-      <c r="A60">
+      <c r="A60" s="2">
         <f>IF(E60="","",COUNTA(E$2:E60))</f>
-        <v/>
       </c>
     </row>
     <row r="61">
-      <c r="A61">
+      <c r="A61" s="2">
         <f>IF(E61="","",COUNTA(E$2:E61))</f>
-        <v/>
       </c>
     </row>
     <row r="62">
-      <c r="A62">
+      <c r="A62" s="2">
         <f>IF(E62="","",COUNTA(E$2:E62))</f>
-        <v/>
       </c>
     </row>
     <row r="63">
-      <c r="A63">
+      <c r="A63" s="2">
         <f>IF(E63="","",COUNTA(E$2:E63))</f>
-        <v/>
       </c>
     </row>
     <row r="64">
-      <c r="A64">
+      <c r="A64" s="2">
         <f>IF(E64="","",COUNTA(E$2:E64))</f>
-        <v/>
       </c>
     </row>
     <row r="65">
-      <c r="A65">
+      <c r="A65" s="2">
         <f>IF(E65="","",COUNTA(E$2:E65))</f>
-        <v/>
       </c>
     </row>
     <row r="66">
-      <c r="A66">
+      <c r="A66" s="2">
         <f>IF(E66="","",COUNTA(E$2:E66))</f>
-        <v/>
       </c>
     </row>
     <row r="67">
-      <c r="A67">
+      <c r="A67" s="2">
         <f>IF(E67="","",COUNTA(E$2:E67))</f>
-        <v/>
       </c>
     </row>
     <row r="68">
-      <c r="A68">
+      <c r="A68" s="2">
         <f>IF(E68="","",COUNTA(E$2:E68))</f>
-        <v/>
       </c>
     </row>
     <row r="69">
-      <c r="A69">
+      <c r="A69" s="2">
         <f>IF(E69="","",COUNTA(E$2:E69))</f>
-        <v/>
       </c>
     </row>
     <row r="70">
-      <c r="A70">
+      <c r="A70" s="2">
         <f>IF(E70="","",COUNTA(E$2:E70))</f>
-        <v/>
       </c>
     </row>
     <row r="71">
-      <c r="A71">
+      <c r="A71" s="2">
         <f>IF(E71="","",COUNTA(E$2:E71))</f>
-        <v/>
       </c>
     </row>
     <row r="72">
-      <c r="A72">
+      <c r="A72" s="2">
         <f>IF(E72="","",COUNTA(E$2:E72))</f>
-        <v/>
       </c>
     </row>
     <row r="73">
-      <c r="A73">
+      <c r="A73" s="2">
         <f>IF(E73="","",COUNTA(E$2:E73))</f>
-        <v/>
       </c>
     </row>
     <row r="74">
-      <c r="A74">
+      <c r="A74" s="2">
         <f>IF(E74="","",COUNTA(E$2:E74))</f>
-        <v/>
       </c>
     </row>
     <row r="75">
-      <c r="A75">
+      <c r="A75" s="2">
         <f>IF(E75="","",COUNTA(E$2:E75))</f>
-        <v/>
       </c>
     </row>
     <row r="76">
-      <c r="A76">
+      <c r="A76" s="2">
         <f>IF(E76="","",COUNTA(E$2:E76))</f>
-        <v/>
       </c>
     </row>
     <row r="77">
-      <c r="A77">
+      <c r="A77" s="2">
         <f>IF(E77="","",COUNTA(E$2:E77))</f>
-        <v/>
       </c>
     </row>
     <row r="78">
-      <c r="A78">
+      <c r="A78" s="2">
         <f>IF(E78="","",COUNTA(E$2:E78))</f>
-        <v/>
       </c>
     </row>
     <row r="79">
-      <c r="A79">
+      <c r="A79" s="2">
         <f>IF(E79="","",COUNTA(E$2:E79))</f>
-        <v/>
       </c>
     </row>
     <row r="80">
-      <c r="A80">
+      <c r="A80" s="2">
         <f>IF(E80="","",COUNTA(E$2:E80))</f>
-        <v/>
       </c>
     </row>
     <row r="81">
-      <c r="A81">
+      <c r="A81" s="2">
         <f>IF(E81="","",COUNTA(E$2:E81))</f>
-        <v/>
       </c>
     </row>
     <row r="82">
-      <c r="A82">
+      <c r="A82" s="2">
         <f>IF(E82="","",COUNTA(E$2:E82))</f>
-        <v/>
       </c>
     </row>
     <row r="83">
-      <c r="A83">
+      <c r="A83" s="2">
         <f>IF(E83="","",COUNTA(E$2:E83))</f>
-        <v/>
       </c>
     </row>
     <row r="84">
-      <c r="A84">
+      <c r="A84" s="2">
         <f>IF(E84="","",COUNTA(E$2:E84))</f>
-        <v/>
       </c>
     </row>
     <row r="85">
-      <c r="A85">
+      <c r="A85" s="2">
         <f>IF(E85="","",COUNTA(E$2:E85))</f>
-        <v/>
       </c>
     </row>
     <row r="86">
-      <c r="A86">
+      <c r="A86" s="2">
         <f>IF(E86="","",COUNTA(E$2:E86))</f>
-        <v/>
       </c>
     </row>
     <row r="87">
-      <c r="A87">
+      <c r="A87" s="2">
         <f>IF(E87="","",COUNTA(E$2:E87))</f>
-        <v/>
       </c>
     </row>
     <row r="88">
-      <c r="A88">
+      <c r="A88" s="2">
         <f>IF(E88="","",COUNTA(E$2:E88))</f>
-        <v/>
       </c>
     </row>
     <row r="89">
-      <c r="A89">
+      <c r="A89" s="2">
         <f>IF(E89="","",COUNTA(E$2:E89))</f>
-        <v/>
       </c>
     </row>
     <row r="90">
-      <c r="A90">
+      <c r="A90" s="2">
         <f>IF(E90="","",COUNTA(E$2:E90))</f>
-        <v/>
       </c>
     </row>
     <row r="91">
-      <c r="A91">
+      <c r="A91" s="2">
         <f>IF(E91="","",COUNTA(E$2:E91))</f>
-        <v/>
       </c>
     </row>
     <row r="92">
-      <c r="A92">
+      <c r="A92" s="2">
         <f>IF(E92="","",COUNTA(E$2:E92))</f>
-        <v/>
       </c>
     </row>
     <row r="93">
-      <c r="A93">
+      <c r="A93" s="2">
         <f>IF(E93="","",COUNTA(E$2:E93))</f>
-        <v/>
       </c>
     </row>
     <row r="94">
-      <c r="A94">
+      <c r="A94" s="2">
         <f>IF(E94="","",COUNTA(E$2:E94))</f>
-        <v/>
       </c>
     </row>
     <row r="95">
-      <c r="A95">
+      <c r="A95" s="2">
         <f>IF(E95="","",COUNTA(E$2:E95))</f>
-        <v/>
       </c>
     </row>
     <row r="96">
-      <c r="A96">
+      <c r="A96" s="2">
         <f>IF(E96="","",COUNTA(E$2:E96))</f>
-        <v/>
       </c>
     </row>
     <row r="97">
-      <c r="A97">
+      <c r="A97" s="2">
         <f>IF(E97="","",COUNTA(E$2:E97))</f>
-        <v/>
       </c>
     </row>
     <row r="98">
-      <c r="A98">
+      <c r="A98" s="2">
         <f>IF(E98="","",COUNTA(E$2:E98))</f>
-        <v/>
       </c>
     </row>
     <row r="99">
-      <c r="A99">
+      <c r="A99" s="2">
         <f>IF(E99="","",COUNTA(E$2:E99))</f>
-        <v/>
       </c>
     </row>
     <row r="100">
-      <c r="A100">
+      <c r="A100" s="2">
         <f>IF(E100="","",COUNTA(E$2:E100))</f>
-        <v/>
       </c>
     </row>
     <row r="101">
-      <c r="A101">
+      <c r="A101" s="2">
         <f>IF(E101="","",COUNTA(E$2:E101))</f>
-        <v/>
       </c>
     </row>
     <row r="102">
-      <c r="A102">
+      <c r="A102" s="2">
         <f>IF(E102="","",COUNTA(E$2:E102))</f>
-        <v/>
       </c>
     </row>
     <row r="103">
-      <c r="A103">
+      <c r="A103" s="2">
         <f>IF(E103="","",COUNTA(E$2:E103))</f>
-        <v/>
       </c>
     </row>
     <row r="104">
-      <c r="A104">
+      <c r="A104" s="2">
         <f>IF(E104="","",COUNTA(E$2:E104))</f>
-        <v/>
       </c>
     </row>
     <row r="105">
-      <c r="A105">
+      <c r="A105" s="2">
         <f>IF(E105="","",COUNTA(E$2:E105))</f>
-        <v/>
       </c>
     </row>
     <row r="106">
-      <c r="A106">
+      <c r="A106" s="2">
         <f>IF(E106="","",COUNTA(E$2:E106))</f>
-        <v/>
       </c>
     </row>
     <row r="107">
-      <c r="A107">
+      <c r="A107" s="2">
         <f>IF(E107="","",COUNTA(E$2:E107))</f>
-        <v/>
       </c>
     </row>
     <row r="108">
-      <c r="A108">
+      <c r="A108" s="2">
         <f>IF(E108="","",COUNTA(E$2:E108))</f>
-        <v/>
       </c>
     </row>
     <row r="109">
-      <c r="A109">
+      <c r="A109" s="2">
         <f>IF(E109="","",COUNTA(E$2:E109))</f>
-        <v/>
       </c>
     </row>
     <row r="110">
-      <c r="A110">
+      <c r="A110" s="2">
         <f>IF(E110="","",COUNTA(E$2:E110))</f>
-        <v/>
       </c>
     </row>
     <row r="111">
-      <c r="A111">
+      <c r="A111" s="2">
         <f>IF(E111="","",COUNTA(E$2:E111))</f>
-        <v/>
       </c>
     </row>
     <row r="112">
-      <c r="A112">
+      <c r="A112" s="2">
         <f>IF(E112="","",COUNTA(E$2:E112))</f>
-        <v/>
       </c>
     </row>
     <row r="113">
-      <c r="A113">
+      <c r="A113" s="2">
         <f>IF(E113="","",COUNTA(E$2:E113))</f>
-        <v/>
       </c>
     </row>
     <row r="114">
-      <c r="A114">
+      <c r="A114" s="2">
         <f>IF(E114="","",COUNTA(E$2:E114))</f>
-        <v/>
       </c>
     </row>
     <row r="115">
-      <c r="A115">
+      <c r="A115" s="2">
         <f>IF(E115="","",COUNTA(E$2:E115))</f>
-        <v/>
       </c>
     </row>
     <row r="116">
-      <c r="A116">
+      <c r="A116" s="2">
         <f>IF(E116="","",COUNTA(E$2:E116))</f>
-        <v/>
       </c>
     </row>
     <row r="117">
-      <c r="A117">
+      <c r="A117" s="2">
         <f>IF(E117="","",COUNTA(E$2:E117))</f>
-        <v/>
       </c>
     </row>
     <row r="118">
-      <c r="A118">
+      <c r="A118" s="2">
         <f>IF(E118="","",COUNTA(E$2:E118))</f>
-        <v/>
       </c>
     </row>
     <row r="119">
-      <c r="A119">
+      <c r="A119" s="2">
         <f>IF(E119="","",COUNTA(E$2:E119))</f>
-        <v/>
       </c>
     </row>
     <row r="120">
-      <c r="A120">
+      <c r="A120" s="2">
         <f>IF(E120="","",COUNTA(E$2:E120))</f>
-        <v/>
       </c>
     </row>
     <row r="121">
-      <c r="A121">
+      <c r="A121" s="2">
         <f>IF(E121="","",COUNTA(E$2:E121))</f>
-        <v/>
       </c>
     </row>
     <row r="122">
-      <c r="A122">
+      <c r="A122" s="2">
         <f>IF(E122="","",COUNTA(E$2:E122))</f>
-        <v/>
       </c>
     </row>
     <row r="123">
-      <c r="A123">
+      <c r="A123" s="2">
         <f>IF(E123="","",COUNTA(E$2:E123))</f>
-        <v/>
       </c>
     </row>
     <row r="124">
-      <c r="A124">
+      <c r="A124" s="2">
         <f>IF(E124="","",COUNTA(E$2:E124))</f>
-        <v/>
       </c>
     </row>
     <row r="125">
-      <c r="A125">
+      <c r="A125" s="2">
         <f>IF(E125="","",COUNTA(E$2:E125))</f>
-        <v/>
       </c>
     </row>
     <row r="126">
-      <c r="A126">
+      <c r="A126" s="2">
         <f>IF(E126="","",COUNTA(E$2:E126))</f>
-        <v/>
       </c>
     </row>
     <row r="127">
-      <c r="A127">
+      <c r="A127" s="2">
         <f>IF(E127="","",COUNTA(E$2:E127))</f>
-        <v/>
       </c>
     </row>
     <row r="128">
-      <c r="A128">
+      <c r="A128" s="2">
         <f>IF(E128="","",COUNTA(E$2:E128))</f>
-        <v/>
       </c>
     </row>
     <row r="129">
-      <c r="A129">
+      <c r="A129" s="2">
         <f>IF(E129="","",COUNTA(E$2:E129))</f>
-        <v/>
       </c>
     </row>
     <row r="130">
-      <c r="A130">
+      <c r="A130" s="2">
         <f>IF(E130="","",COUNTA(E$2:E130))</f>
-        <v/>
       </c>
     </row>
     <row r="131">
-      <c r="A131">
+      <c r="A131" s="2">
         <f>IF(E131="","",COUNTA(E$2:E131))</f>
-        <v/>
       </c>
     </row>
     <row r="132">
-      <c r="A132">
+      <c r="A132" s="2">
         <f>IF(E132="","",COUNTA(E$2:E132))</f>
-        <v/>
       </c>
     </row>
     <row r="133">
-      <c r="A133">
+      <c r="A133" s="2">
         <f>IF(E133="","",COUNTA(E$2:E133))</f>
-        <v/>
       </c>
     </row>
     <row r="134">
-      <c r="A134">
+      <c r="A134" s="2">
         <f>IF(E134="","",COUNTA(E$2:E134))</f>
-        <v/>
       </c>
     </row>
     <row r="135">
-      <c r="A135">
+      <c r="A135" s="2">
         <f>IF(E135="","",COUNTA(E$2:E135))</f>
-        <v/>
       </c>
     </row>
     <row r="136">
-      <c r="A136">
+      <c r="A136" s="2">
         <f>IF(E136="","",COUNTA(E$2:E136))</f>
-        <v/>
       </c>
     </row>
     <row r="137">
-      <c r="A137">
+      <c r="A137" s="2">
         <f>IF(E137="","",COUNTA(E$2:E137))</f>
-        <v/>
       </c>
     </row>
     <row r="138">
-      <c r="A138">
+      <c r="A138" s="2">
         <f>IF(E138="","",COUNTA(E$2:E138))</f>
-        <v/>
       </c>
     </row>
     <row r="139">
-      <c r="A139">
+      <c r="A139" s="2">
         <f>IF(E139="","",COUNTA(E$2:E139))</f>
-        <v/>
       </c>
     </row>
     <row r="140">
-      <c r="A140">
+      <c r="A140" s="2">
         <f>IF(E140="","",COUNTA(E$2:E140))</f>
-        <v/>
       </c>
     </row>
     <row r="141">
-      <c r="A141">
+      <c r="A141" s="2">
         <f>IF(E141="","",COUNTA(E$2:E141))</f>
-        <v/>
       </c>
     </row>
     <row r="142">
-      <c r="A142">
+      <c r="A142" s="2">
         <f>IF(E142="","",COUNTA(E$2:E142))</f>
-        <v/>
       </c>
     </row>
     <row r="143">
-      <c r="A143">
+      <c r="A143" s="2">
         <f>IF(E143="","",COUNTA(E$2:E143))</f>
-        <v/>
       </c>
     </row>
     <row r="144">
-      <c r="A144">
+      <c r="A144" s="2">
         <f>IF(E144="","",COUNTA(E$2:E144))</f>
-        <v/>
       </c>
     </row>
     <row r="145">
-      <c r="A145">
+      <c r="A145" s="2">
         <f>IF(E145="","",COUNTA(E$2:E145))</f>
-        <v/>
       </c>
     </row>
     <row r="146">
-      <c r="A146">
+      <c r="A146" s="2">
         <f>IF(E146="","",COUNTA(E$2:E146))</f>
-        <v/>
       </c>
     </row>
     <row r="147">
-      <c r="A147">
+      <c r="A147" s="2">
         <f>IF(E147="","",COUNTA(E$2:E147))</f>
-        <v/>
       </c>
     </row>
     <row r="148">
-      <c r="A148">
+      <c r="A148" s="2">
         <f>IF(E148="","",COUNTA(E$2:E148))</f>
-        <v/>
       </c>
     </row>
     <row r="149">
-      <c r="A149">
+      <c r="A149" s="2">
         <f>IF(E149="","",COUNTA(E$2:E149))</f>
-        <v/>
       </c>
     </row>
     <row r="150">
-      <c r="A150">
+      <c r="A150" s="2">
         <f>IF(E150="","",COUNTA(E$2:E150))</f>
-        <v/>
       </c>
     </row>
     <row r="151">
-      <c r="A151">
+      <c r="A151" s="2">
         <f>IF(E151="","",COUNTA(E$2:E151))</f>
-        <v/>
       </c>
     </row>
     <row r="152">
-      <c r="A152">
+      <c r="A152" s="2">
         <f>IF(E152="","",COUNTA(E$2:E152))</f>
-        <v/>
       </c>
     </row>
     <row r="153">
-      <c r="A153">
+      <c r="A153" s="2">
         <f>IF(E153="","",COUNTA(E$2:E153))</f>
-        <v/>
       </c>
     </row>
     <row r="154">
-      <c r="A154">
+      <c r="A154" s="2">
         <f>IF(E154="","",COUNTA(E$2:E154))</f>
-        <v/>
       </c>
     </row>
     <row r="155">
-      <c r="A155">
+      <c r="A155" s="2">
         <f>IF(E155="","",COUNTA(E$2:E155))</f>
-        <v/>
       </c>
     </row>
     <row r="156">
-      <c r="A156">
+      <c r="A156" s="2">
         <f>IF(E156="","",COUNTA(E$2:E156))</f>
-        <v/>
       </c>
     </row>
     <row r="157">
-      <c r="A157">
+      <c r="A157" s="2">
         <f>IF(E157="","",COUNTA(E$2:E157))</f>
-        <v/>
       </c>
     </row>
     <row r="158">
-      <c r="A158">
+      <c r="A158" s="2">
         <f>IF(E158="","",COUNTA(E$2:E158))</f>
-        <v/>
       </c>
     </row>
     <row r="159">
-      <c r="A159">
+      <c r="A159" s="2">
         <f>IF(E159="","",COUNTA(E$2:E159))</f>
-        <v/>
       </c>
     </row>
     <row r="160">
-      <c r="A160">
+      <c r="A160" s="2">
         <f>IF(E160="","",COUNTA(E$2:E160))</f>
-        <v/>
       </c>
     </row>
     <row r="161">
-      <c r="A161">
+      <c r="A161" s="2">
         <f>IF(E161="","",COUNTA(E$2:E161))</f>
-        <v/>
       </c>
     </row>
     <row r="162">
-      <c r="A162">
+      <c r="A162" s="2">
         <f>IF(E162="","",COUNTA(E$2:E162))</f>
-        <v/>
       </c>
     </row>
     <row r="163">
-      <c r="A163">
+      <c r="A163" s="2">
         <f>IF(E163="","",COUNTA(E$2:E163))</f>
-        <v/>
       </c>
     </row>
     <row r="164">
-      <c r="A164">
+      <c r="A164" s="2">
         <f>IF(E164="","",COUNTA(E$2:E164))</f>
-        <v/>
       </c>
     </row>
     <row r="165">
-      <c r="A165">
+      <c r="A165" s="2">
         <f>IF(E165="","",COUNTA(E$2:E165))</f>
-        <v/>
       </c>
     </row>
     <row r="166">
-      <c r="A166">
+      <c r="A166" s="2">
         <f>IF(E166="","",COUNTA(E$2:E166))</f>
-        <v/>
       </c>
     </row>
     <row r="167">
-      <c r="A167">
+      <c r="A167" s="2">
         <f>IF(E167="","",COUNTA(E$2:E167))</f>
-        <v/>
       </c>
     </row>
     <row r="168">
-      <c r="A168">
+      <c r="A168" s="2">
         <f>IF(E168="","",COUNTA(E$2:E168))</f>
-        <v/>
       </c>
     </row>
     <row r="169">
-      <c r="A169">
+      <c r="A169" s="2">
         <f>IF(E169="","",COUNTA(E$2:E169))</f>
-        <v/>
       </c>
     </row>
     <row r="170">
-      <c r="A170">
+      <c r="A170" s="2">
         <f>IF(E170="","",COUNTA(E$2:E170))</f>
-        <v/>
       </c>
     </row>
     <row r="171">
-      <c r="A171">
+      <c r="A171" s="2">
         <f>IF(E171="","",COUNTA(E$2:E171))</f>
-        <v/>
       </c>
     </row>
     <row r="172">
-      <c r="A172">
+      <c r="A172" s="2">
         <f>IF(E172="","",COUNTA(E$2:E172))</f>
-        <v/>
       </c>
     </row>
     <row r="173">
-      <c r="A173">
+      <c r="A173" s="2">
         <f>IF(E173="","",COUNTA(E$2:E173))</f>
-        <v/>
       </c>
     </row>
     <row r="174">
-      <c r="A174">
+      <c r="A174" s="2">
         <f>IF(E174="","",COUNTA(E$2:E174))</f>
-        <v/>
       </c>
     </row>
     <row r="175">
-      <c r="A175">
+      <c r="A175" s="2">
         <f>IF(E175="","",COUNTA(E$2:E175))</f>
-        <v/>
       </c>
     </row>
     <row r="176">
-      <c r="A176">
+      <c r="A176" s="2">
         <f>IF(E176="","",COUNTA(E$2:E176))</f>
-        <v/>
       </c>
     </row>
     <row r="177">
-      <c r="A177">
+      <c r="A177" s="2">
         <f>IF(E177="","",COUNTA(E$2:E177))</f>
-        <v/>
       </c>
     </row>
     <row r="178">
-      <c r="A178">
+      <c r="A178" s="2">
         <f>IF(E178="","",COUNTA(E$2:E178))</f>
-        <v/>
       </c>
     </row>
     <row r="179">
-      <c r="A179">
+      <c r="A179" s="2">
         <f>IF(E179="","",COUNTA(E$2:E179))</f>
-        <v/>
       </c>
     </row>
     <row r="180">
-      <c r="A180">
+      <c r="A180" s="2">
         <f>IF(E180="","",COUNTA(E$2:E180))</f>
-        <v/>
       </c>
     </row>
     <row r="181">
-      <c r="A181">
+      <c r="A181" s="2">
         <f>IF(E181="","",COUNTA(E$2:E181))</f>
-        <v/>
       </c>
     </row>
     <row r="182">
-      <c r="A182">
+      <c r="A182" s="2">
         <f>IF(E182="","",COUNTA(E$2:E182))</f>
-        <v/>
       </c>
     </row>
     <row r="183">
-      <c r="A183">
+      <c r="A183" s="2">
         <f>IF(E183="","",COUNTA(E$2:E183))</f>
-        <v/>
       </c>
     </row>
     <row r="184">
-      <c r="A184">
+      <c r="A184" s="2">
         <f>IF(E184="","",COUNTA(E$2:E184))</f>
-        <v/>
       </c>
     </row>
     <row r="185">
-      <c r="A185">
+      <c r="A185" s="2">
         <f>IF(E185="","",COUNTA(E$2:E185))</f>
-        <v/>
       </c>
     </row>
     <row r="186">
-      <c r="A186">
+      <c r="A186" s="2">
         <f>IF(E186="","",COUNTA(E$2:E186))</f>
-        <v/>
       </c>
     </row>
     <row r="187">
-      <c r="A187">
+      <c r="A187" s="2">
         <f>IF(E187="","",COUNTA(E$2:E187))</f>
-        <v/>
       </c>
     </row>
     <row r="188">
-      <c r="A188">
+      <c r="A188" s="2">
         <f>IF(E188="","",COUNTA(E$2:E188))</f>
-        <v/>
       </c>
     </row>
     <row r="189">
-      <c r="A189">
+      <c r="A189" s="2">
         <f>IF(E189="","",COUNTA(E$2:E189))</f>
-        <v/>
       </c>
     </row>
     <row r="190">
-      <c r="A190">
+      <c r="A190" s="2">
         <f>IF(E190="","",COUNTA(E$2:E190))</f>
-        <v/>
       </c>
     </row>
     <row r="191">
-      <c r="A191">
+      <c r="A191" s="2">
         <f>IF(E191="","",COUNTA(E$2:E191))</f>
-        <v/>
       </c>
     </row>
     <row r="192">
-      <c r="A192">
+      <c r="A192" s="2">
         <f>IF(E192="","",COUNTA(E$2:E192))</f>
-        <v/>
       </c>
     </row>
     <row r="193">
-      <c r="A193">
+      <c r="A193" s="2">
         <f>IF(E193="","",COUNTA(E$2:E193))</f>
-        <v/>
       </c>
     </row>
     <row r="194">
-      <c r="A194">
+      <c r="A194" s="2">
         <f>IF(E194="","",COUNTA(E$2:E194))</f>
-        <v/>
       </c>
     </row>
     <row r="195">
-      <c r="A195">
+      <c r="A195" s="2">
         <f>IF(E195="","",COUNTA(E$2:E195))</f>
-        <v/>
       </c>
     </row>
     <row r="196">
-      <c r="A196">
+      <c r="A196" s="2">
         <f>IF(E196="","",COUNTA(E$2:E196))</f>
-        <v/>
       </c>
     </row>
     <row r="197">
-      <c r="A197">
+      <c r="A197" s="2">
         <f>IF(E197="","",COUNTA(E$2:E197))</f>
-        <v/>
       </c>
     </row>
     <row r="198">
-      <c r="A198">
+      <c r="A198" s="2">
         <f>IF(E198="","",COUNTA(E$2:E198))</f>
-        <v/>
       </c>
     </row>
     <row r="199">
-      <c r="A199">
+      <c r="A199" s="2">
         <f>IF(E199="","",COUNTA(E$2:E199))</f>
-        <v/>
       </c>
     </row>
     <row r="200">
-      <c r="A200">
+      <c r="A200" s="2">
         <f>IF(E200="","",COUNTA(E$2:E200))</f>
-        <v/>
       </c>
     </row>
     <row r="201">
-      <c r="A201">
+      <c r="A201" s="2">
         <f>IF(E201="","",COUNTA(E$2:E201))</f>
-        <v/>
       </c>
     </row>
     <row r="202">
-      <c r="A202">
+      <c r="A202" s="2">
         <f>IF(E202="","",COUNTA(E$2:E202))</f>
-        <v/>
       </c>
     </row>
     <row r="203">
-      <c r="A203">
+      <c r="A203" s="2">
         <f>IF(E203="","",COUNTA(E$2:E203))</f>
-        <v/>
       </c>
     </row>
     <row r="204">
-      <c r="A204">
+      <c r="A204" s="2">
         <f>IF(E204="","",COUNTA(E$2:E204))</f>
-        <v/>
       </c>
     </row>
     <row r="205">
-      <c r="A205">
+      <c r="A205" s="2">
         <f>IF(E205="","",COUNTA(E$2:E205))</f>
-        <v/>
       </c>
     </row>
     <row r="206">
-      <c r="A206">
+      <c r="A206" s="2">
         <f>IF(E206="","",COUNTA(E$2:E206))</f>
-        <v/>
       </c>
     </row>
     <row r="207">
-      <c r="A207">
+      <c r="A207" s="2">
         <f>IF(E207="","",COUNTA(E$2:E207))</f>
-        <v/>
       </c>
     </row>
     <row r="208">
-      <c r="A208">
+      <c r="A208" s="2">
         <f>IF(E208="","",COUNTA(E$2:E208))</f>
-        <v/>
       </c>
     </row>
     <row r="209">
-      <c r="A209">
+      <c r="A209" s="2">
         <f>IF(E209="","",COUNTA(E$2:E209))</f>
-        <v/>
       </c>
     </row>
     <row r="210">
-      <c r="A210">
+      <c r="A210" s="2">
         <f>IF(E210="","",COUNTA(E$2:E210))</f>
-        <v/>
       </c>
     </row>
     <row r="211">
-      <c r="A211">
+      <c r="A211" s="2">
         <f>IF(E211="","",COUNTA(E$2:E211))</f>
-        <v/>
       </c>
     </row>
     <row r="212">
-      <c r="A212">
+      <c r="A212" s="2">
         <f>IF(E212="","",COUNTA(E$2:E212))</f>
-        <v/>
       </c>
     </row>
     <row r="213">
-      <c r="A213">
+      <c r="A213" s="2">
         <f>IF(E213="","",COUNTA(E$2:E213))</f>
-        <v/>
       </c>
     </row>
     <row r="214">
-      <c r="A214">
+      <c r="A214" s="2">
         <f>IF(E214="","",COUNTA(E$2:E214))</f>
-        <v/>
       </c>
     </row>
     <row r="215">
-      <c r="A215">
+      <c r="A215" s="2">
         <f>IF(E215="","",COUNTA(E$2:E215))</f>
-        <v/>
       </c>
     </row>
     <row r="216">
-      <c r="A216">
+      <c r="A216" s="2">
         <f>IF(E216="","",COUNTA(E$2:E216))</f>
-        <v/>
       </c>
     </row>
     <row r="217">
-      <c r="A217">
+      <c r="A217" s="2">
         <f>IF(E217="","",COUNTA(E$2:E217))</f>
-        <v/>
       </c>
     </row>
     <row r="218">
-      <c r="A218">
+      <c r="A218" s="2">
         <f>IF(E218="","",COUNTA(E$2:E218))</f>
-        <v/>
       </c>
     </row>
     <row r="219">
-      <c r="A219">
+      <c r="A219" s="2">
         <f>IF(E219="","",COUNTA(E$2:E219))</f>
-        <v/>
       </c>
     </row>
     <row r="220">
-      <c r="A220">
+      <c r="A220" s="2">
         <f>IF(E220="","",COUNTA(E$2:E220))</f>
-        <v/>
       </c>
     </row>
     <row r="221">
-      <c r="A221">
+      <c r="A221" s="2">
         <f>IF(E221="","",COUNTA(E$2:E221))</f>
-        <v/>
       </c>
     </row>
     <row r="222">
-      <c r="A222">
+      <c r="A222" s="2">
         <f>IF(E222="","",COUNTA(E$2:E222))</f>
-        <v/>
       </c>
     </row>
     <row r="223">
-      <c r="A223">
+      <c r="A223" s="2">
         <f>IF(E223="","",COUNTA(E$2:E223))</f>
-        <v/>
       </c>
     </row>
     <row r="224">
-      <c r="A224">
+      <c r="A224" s="2">
         <f>IF(E224="","",COUNTA(E$2:E224))</f>
-        <v/>
       </c>
     </row>
     <row r="225">
-      <c r="A225">
+      <c r="A225" s="2">
         <f>IF(E225="","",COUNTA(E$2:E225))</f>
-        <v/>
       </c>
     </row>
     <row r="226">
-      <c r="A226">
+      <c r="A226" s="2">
         <f>IF(E226="","",COUNTA(E$2:E226))</f>
-        <v/>
       </c>
     </row>
     <row r="227">
-      <c r="A227">
+      <c r="A227" s="2">
         <f>IF(E227="","",COUNTA(E$2:E227))</f>
-        <v/>
       </c>
     </row>
     <row r="228">
-      <c r="A228">
+      <c r="A228" s="2">
         <f>IF(E228="","",COUNTA(E$2:E228))</f>
-        <v/>
       </c>
     </row>
     <row r="229">
-      <c r="A229">
+      <c r="A229" s="2">
         <f>IF(E229="","",COUNTA(E$2:E229))</f>
-        <v/>
       </c>
     </row>
     <row r="230">
-      <c r="A230">
+      <c r="A230" s="2">
         <f>IF(E230="","",COUNTA(E$2:E230))</f>
-        <v/>
       </c>
     </row>
     <row r="231">
-      <c r="A231">
+      <c r="A231" s="2">
         <f>IF(E231="","",COUNTA(E$2:E231))</f>
-        <v/>
       </c>
     </row>
     <row r="232">
-      <c r="A232">
+      <c r="A232" s="2">
         <f>IF(E232="","",COUNTA(E$2:E232))</f>
-        <v/>
       </c>
     </row>
     <row r="233">
-      <c r="A233">
+      <c r="A233" s="2">
         <f>IF(E233="","",COUNTA(E$2:E233))</f>
-        <v/>
       </c>
     </row>
     <row r="234">
-      <c r="A234">
+      <c r="A234" s="2">
         <f>IF(E234="","",COUNTA(E$2:E234))</f>
-        <v/>
       </c>
     </row>
     <row r="235">
-      <c r="A235">
+      <c r="A235" s="2">
         <f>IF(E235="","",COUNTA(E$2:E235))</f>
-        <v/>
       </c>
     </row>
     <row r="236">
-      <c r="A236">
+      <c r="A236" s="2">
         <f>IF(E236="","",COUNTA(E$2:E236))</f>
-        <v/>
       </c>
     </row>
     <row r="237">
-      <c r="A237">
+      <c r="A237" s="2">
         <f>IF(E237="","",COUNTA(E$2:E237))</f>
-        <v/>
       </c>
     </row>
     <row r="238">
-      <c r="A238">
+      <c r="A238" s="2">
         <f>IF(E238="","",COUNTA(E$2:E238))</f>
-        <v/>
       </c>
     </row>
     <row r="239">
-      <c r="A239">
+      <c r="A239" s="2">
         <f>IF(E239="","",COUNTA(E$2:E239))</f>
-        <v/>
       </c>
     </row>
     <row r="240">
-      <c r="A240">
+      <c r="A240" s="2">
         <f>IF(E240="","",COUNTA(E$2:E240))</f>
-        <v/>
       </c>
     </row>
     <row r="241">
-      <c r="A241">
+      <c r="A241" s="2">
         <f>IF(E241="","",COUNTA(E$2:E241))</f>
-        <v/>
       </c>
     </row>
     <row r="242">
-      <c r="A242">
+      <c r="A242" s="2">
         <f>IF(E242="","",COUNTA(E$2:E242))</f>
-        <v/>
       </c>
     </row>
     <row r="243">
-      <c r="A243">
+      <c r="A243" s="2">
         <f>IF(E243="","",COUNTA(E$2:E243))</f>
-        <v/>
       </c>
     </row>
     <row r="244">
-      <c r="A244">
+      <c r="A244" s="2">
         <f>IF(E244="","",COUNTA(E$2:E244))</f>
-        <v/>
       </c>
     </row>
     <row r="245">
-      <c r="A245">
+      <c r="A245" s="2">
         <f>IF(E245="","",COUNTA(E$2:E245))</f>
-        <v/>
       </c>
     </row>
     <row r="246">
-      <c r="A246">
+      <c r="A246" s="2">
         <f>IF(E246="","",COUNTA(E$2:E246))</f>
-        <v/>
       </c>
     </row>
     <row r="247">
-      <c r="A247">
+      <c r="A247" s="2">
         <f>IF(E247="","",COUNTA(E$2:E247))</f>
-        <v/>
       </c>
     </row>
     <row r="248">
-      <c r="A248">
+      <c r="A248" s="2">
         <f>IF(E248="","",COUNTA(E$2:E248))</f>
-        <v/>
       </c>
     </row>
     <row r="249">
-      <c r="A249">
+      <c r="A249" s="2">
         <f>IF(E249="","",COUNTA(E$2:E249))</f>
-        <v/>
       </c>
     </row>
     <row r="250">
-      <c r="A250">
+      <c r="A250" s="2">
         <f>IF(E250="","",COUNTA(E$2:E250))</f>
-        <v/>
       </c>
     </row>
     <row r="251">
-      <c r="A251">
+      <c r="A251" s="2">
         <f>IF(E251="","",COUNTA(E$2:E251))</f>
-        <v/>
       </c>
     </row>
     <row r="252">
-      <c r="A252">
+      <c r="A252" s="2">
         <f>IF(E252="","",COUNTA(E$2:E252))</f>
-        <v/>
       </c>
     </row>
     <row r="253">
-      <c r="A253">
+      <c r="A253" s="2">
         <f>IF(E253="","",COUNTA(E$2:E253))</f>
-        <v/>
       </c>
     </row>
     <row r="254">
-      <c r="A254">
+      <c r="A254" s="2">
         <f>IF(E254="","",COUNTA(E$2:E254))</f>
-        <v/>
       </c>
     </row>
     <row r="255">
-      <c r="A255">
+      <c r="A255" s="2">
         <f>IF(E255="","",COUNTA(E$2:E255))</f>
-        <v/>
       </c>
     </row>
     <row r="256">
-      <c r="A256">
+      <c r="A256" s="2">
         <f>IF(E256="","",COUNTA(E$2:E256))</f>
-        <v/>
       </c>
     </row>
     <row r="257">
-      <c r="A257">
+      <c r="A257" s="2">
         <f>IF(E257="","",COUNTA(E$2:E257))</f>
-        <v/>
       </c>
     </row>
     <row r="258">
-      <c r="A258">
+      <c r="A258" s="2">
         <f>IF(E258="","",COUNTA(E$2:E258))</f>
-        <v/>
       </c>
     </row>
     <row r="259">
-      <c r="A259">
+      <c r="A259" s="2">
         <f>IF(E259="","",COUNTA(E$2:E259))</f>
-        <v/>
       </c>
     </row>
     <row r="260">
-      <c r="A260">
+      <c r="A260" s="2">
         <f>IF(E260="","",COUNTA(E$2:E260))</f>
-        <v/>
       </c>
     </row>
     <row r="261">
-      <c r="A261">
+      <c r="A261" s="2">
         <f>IF(E261="","",COUNTA(E$2:E261))</f>
-        <v/>
       </c>
     </row>
     <row r="262">
-      <c r="A262">
+      <c r="A262" s="2">
         <f>IF(E262="","",COUNTA(E$2:E262))</f>
-        <v/>
       </c>
     </row>
     <row r="263">
-      <c r="A263">
+      <c r="A263" s="2">
         <f>IF(E263="","",COUNTA(E$2:E263))</f>
-        <v/>
       </c>
     </row>
     <row r="264">
-      <c r="A264">
+      <c r="A264" s="2">
         <f>IF(E264="","",COUNTA(E$2:E264))</f>
-        <v/>
       </c>
     </row>
     <row r="265">
-      <c r="A265">
+      <c r="A265" s="2">
         <f>IF(E265="","",COUNTA(E$2:E265))</f>
-        <v/>
       </c>
     </row>
     <row r="266">
-      <c r="A266">
+      <c r="A266" s="2">
         <f>IF(E266="","",COUNTA(E$2:E266))</f>
-        <v/>
       </c>
     </row>
     <row r="267">
-      <c r="A267">
+      <c r="A267" s="2">
         <f>IF(E267="","",COUNTA(E$2:E267))</f>
-        <v/>
       </c>
     </row>
     <row r="268">
-      <c r="A268">
+      <c r="A268" s="2">
         <f>IF(E268="","",COUNTA(E$2:E268))</f>
-        <v/>
       </c>
     </row>
     <row r="269">
-      <c r="A269">
+      <c r="A269" s="2">
         <f>IF(E269="","",COUNTA(E$2:E269))</f>
-        <v/>
       </c>
     </row>
     <row r="270">
-      <c r="A270">
+      <c r="A270" s="2">
         <f>IF(E270="","",COUNTA(E$2:E270))</f>
-        <v/>
       </c>
     </row>
     <row r="271">
-      <c r="A271">
+      <c r="A271" s="2">
         <f>IF(E271="","",COUNTA(E$2:E271))</f>
-        <v/>
       </c>
     </row>
     <row r="272">
-      <c r="A272">
+      <c r="A272" s="2">
         <f>IF(E272="","",COUNTA(E$2:E272))</f>
-        <v/>
       </c>
     </row>
     <row r="273">
-      <c r="A273">
+      <c r="A273" s="2">
         <f>IF(E273="","",COUNTA(E$2:E273))</f>
-        <v/>
       </c>
     </row>
     <row r="274">
-      <c r="A274">
+      <c r="A274" s="2">
         <f>IF(E274="","",COUNTA(E$2:E274))</f>
-        <v/>
       </c>
     </row>
     <row r="275">
-      <c r="A275">
+      <c r="A275" s="2">
         <f>IF(E275="","",COUNTA(E$2:E275))</f>
-        <v/>
       </c>
     </row>
     <row r="276">
-      <c r="A276">
+      <c r="A276" s="2">
         <f>IF(E276="","",COUNTA(E$2:E276))</f>
-        <v/>
       </c>
     </row>
     <row r="277">
-      <c r="A277">
+      <c r="A277" s="2">
         <f>IF(E277="","",COUNTA(E$2:E277))</f>
-        <v/>
       </c>
     </row>
     <row r="278">
-      <c r="A278">
+      <c r="A278" s="2">
         <f>IF(E278="","",COUNTA(E$2:E278))</f>
-        <v/>
       </c>
     </row>
     <row r="279">
-      <c r="A279">
+      <c r="A279" s="2">
         <f>IF(E279="","",COUNTA(E$2:E279))</f>
-        <v/>
       </c>
     </row>
     <row r="280">
-      <c r="A280">
+      <c r="A280" s="2">
         <f>IF(E280="","",COUNTA(E$2:E280))</f>
-        <v/>
       </c>
     </row>
     <row r="281">
-      <c r="A281">
+      <c r="A281" s="2">
         <f>IF(E281="","",COUNTA(E$2:E281))</f>
-        <v/>
       </c>
     </row>
     <row r="282">
-      <c r="A282">
+      <c r="A282" s="2">
         <f>IF(E282="","",COUNTA(E$2:E282))</f>
-        <v/>
       </c>
     </row>
     <row r="283">
-      <c r="A283">
+      <c r="A283" s="2">
         <f>IF(E283="","",COUNTA(E$2:E283))</f>
-        <v/>
       </c>
     </row>
     <row r="284">
-      <c r="A284">
+      <c r="A284" s="2">
         <f>IF(E284="","",COUNTA(E$2:E284))</f>
-        <v/>
       </c>
     </row>
     <row r="285">
-      <c r="A285">
+      <c r="A285" s="2">
         <f>IF(E285="","",COUNTA(E$2:E285))</f>
-        <v/>
       </c>
     </row>
     <row r="286">
-      <c r="A286">
+      <c r="A286" s="2">
         <f>IF(E286="","",COUNTA(E$2:E286))</f>
-        <v/>
       </c>
     </row>
     <row r="287">
-      <c r="A287">
+      <c r="A287" s="2">
         <f>IF(E287="","",COUNTA(E$2:E287))</f>
-        <v/>
       </c>
     </row>
     <row r="288">
-      <c r="A288">
+      <c r="A288" s="2">
         <f>IF(E288="","",COUNTA(E$2:E288))</f>
-        <v/>
       </c>
     </row>
     <row r="289">
-      <c r="A289">
+      <c r="A289" s="2">
         <f>IF(E289="","",COUNTA(E$2:E289))</f>
-        <v/>
       </c>
     </row>
     <row r="290">
-      <c r="A290">
+      <c r="A290" s="2">
         <f>IF(E290="","",COUNTA(E$2:E290))</f>
-        <v/>
       </c>
     </row>
     <row r="291">
-      <c r="A291">
+      <c r="A291" s="2">
         <f>IF(E291="","",COUNTA(E$2:E291))</f>
-        <v/>
       </c>
     </row>
     <row r="292">
-      <c r="A292">
+      <c r="A292" s="2">
         <f>IF(E292="","",COUNTA(E$2:E292))</f>
-        <v/>
       </c>
     </row>
     <row r="293">
-      <c r="A293">
+      <c r="A293" s="2">
         <f>IF(E293="","",COUNTA(E$2:E293))</f>
-        <v/>
       </c>
     </row>
     <row r="294">
-      <c r="A294">
+      <c r="A294" s="2">
         <f>IF(E294="","",COUNTA(E$2:E294))</f>
-        <v/>
       </c>
     </row>
     <row r="295">
-      <c r="A295">
+      <c r="A295" s="2">
         <f>IF(E295="","",COUNTA(E$2:E295))</f>
-        <v/>
       </c>
     </row>
     <row r="296">
-      <c r="A296">
+      <c r="A296" s="2">
         <f>IF(E296="","",COUNTA(E$2:E296))</f>
-        <v/>
       </c>
     </row>
     <row r="297">
-      <c r="A297">
+      <c r="A297" s="2">
         <f>IF(E297="","",COUNTA(E$2:E297))</f>
-        <v/>
       </c>
     </row>
     <row r="298">
-      <c r="A298">
+      <c r="A298" s="2">
         <f>IF(E298="","",COUNTA(E$2:E298))</f>
-        <v/>
       </c>
     </row>
     <row r="299">
-      <c r="A299">
+      <c r="A299" s="2">
         <f>IF(E299="","",COUNTA(E$2:E299))</f>
-        <v/>
       </c>
     </row>
     <row r="300">
-      <c r="A300">
+      <c r="A300" s="2">
         <f>IF(E300="","",COUNTA(E$2:E300))</f>
-        <v/>
       </c>
     </row>
     <row r="301">
-      <c r="A301">
+      <c r="A301" s="2">
         <f>IF(E301="","",COUNTA(E$2:E301))</f>
-        <v/>
       </c>
     </row>
     <row r="302">
-      <c r="A302">
+      <c r="A302" s="2">
         <f>IF(E302="","",COUNTA(E$2:E302))</f>
-        <v/>
       </c>
     </row>
     <row r="303">
-      <c r="A303">
+      <c r="A303" s="2">
         <f>IF(E303="","",COUNTA(E$2:E303))</f>
-        <v/>
       </c>
     </row>
     <row r="304">
-      <c r="A304">
+      <c r="A304" s="2">
         <f>IF(E304="","",COUNTA(E$2:E304))</f>
-        <v/>
       </c>
     </row>
     <row r="305">
-      <c r="A305">
+      <c r="A305" s="2">
         <f>IF(E305="","",COUNTA(E$2:E305))</f>
-        <v/>
       </c>
     </row>
     <row r="306">
-      <c r="A306">
+      <c r="A306" s="2">
         <f>IF(E306="","",COUNTA(E$2:E306))</f>
-        <v/>
       </c>
     </row>
     <row r="307">
-      <c r="A307">
+      <c r="A307" s="2">
         <f>IF(E307="","",COUNTA(E$2:E307))</f>
-        <v/>
       </c>
     </row>
     <row r="308">
-      <c r="A308">
+      <c r="A308" s="2">
         <f>IF(E308="","",COUNTA(E$2:E308))</f>
-        <v/>
       </c>
     </row>
     <row r="309">
-      <c r="A309">
+      <c r="A309" s="2">
         <f>IF(E309="","",COUNTA(E$2:E309))</f>
-        <v/>
       </c>
     </row>
     <row r="310">
-      <c r="A310">
+      <c r="A310" s="2">
         <f>IF(E310="","",COUNTA(E$2:E310))</f>
-        <v/>
       </c>
     </row>
     <row r="311">
-      <c r="A311">
+      <c r="A311" s="2">
         <f>IF(E311="","",COUNTA(E$2:E311))</f>
-        <v/>
       </c>
     </row>
     <row r="312">
-      <c r="A312">
+      <c r="A312" s="2">
         <f>IF(E312="","",COUNTA(E$2:E312))</f>
-        <v/>
       </c>
     </row>
     <row r="313">
-      <c r="A313">
+      <c r="A313" s="2">
         <f>IF(E313="","",COUNTA(E$2:E313))</f>
-        <v/>
       </c>
     </row>
     <row r="314">
-      <c r="A314">
+      <c r="A314" s="2">
         <f>IF(E314="","",COUNTA(E$2:E314))</f>
-        <v/>
       </c>
     </row>
     <row r="315">
-      <c r="A315">
+      <c r="A315" s="2">
         <f>IF(E315="","",COUNTA(E$2:E315))</f>
-        <v/>
       </c>
     </row>
     <row r="316">
-      <c r="A316">
+      <c r="A316" s="2">
         <f>IF(E316="","",COUNTA(E$2:E316))</f>
-        <v/>
       </c>
     </row>
     <row r="317">
-      <c r="A317">
+      <c r="A317" s="2">
         <f>IF(E317="","",COUNTA(E$2:E317))</f>
-        <v/>
       </c>
     </row>
     <row r="318">
-      <c r="A318">
+      <c r="A318" s="2">
         <f>IF(E318="","",COUNTA(E$2:E318))</f>
-        <v/>
       </c>
     </row>
     <row r="319">
-      <c r="A319">
+      <c r="A319" s="2">
         <f>IF(E319="","",COUNTA(E$2:E319))</f>
-        <v/>
       </c>
     </row>
     <row r="320">
-      <c r="A320">
+      <c r="A320" s="2">
         <f>IF(E320="","",COUNTA(E$2:E320))</f>
-        <v/>
       </c>
     </row>
     <row r="321">
-      <c r="A321">
+      <c r="A321" s="2">
         <f>IF(E321="","",COUNTA(E$2:E321))</f>
-        <v/>
       </c>
     </row>
     <row r="322">
-      <c r="A322">
+      <c r="A322" s="2">
         <f>IF(E322="","",COUNTA(E$2:E322))</f>
-        <v/>
       </c>
     </row>
     <row r="323">
-      <c r="A323">
+      <c r="A323" s="2">
         <f>IF(E323="","",COUNTA(E$2:E323))</f>
-        <v/>
       </c>
     </row>
     <row r="324">
-      <c r="A324">
+      <c r="A324" s="2">
         <f>IF(E324="","",COUNTA(E$2:E324))</f>
-        <v/>
       </c>
     </row>
     <row r="325">
-      <c r="A325">
+      <c r="A325" s="2">
         <f>IF(E325="","",COUNTA(E$2:E325))</f>
-        <v/>
       </c>
     </row>
     <row r="326">
-      <c r="A326">
+      <c r="A326" s="2">
         <f>IF(E326="","",COUNTA(E$2:E326))</f>
-        <v/>
       </c>
     </row>
     <row r="327">
-      <c r="A327">
+      <c r="A327" s="2">
         <f>IF(E327="","",COUNTA(E$2:E327))</f>
-        <v/>
       </c>
     </row>
     <row r="328">
-      <c r="A328">
+      <c r="A328" s="2">
         <f>IF(E328="","",COUNTA(E$2:E328))</f>
-        <v/>
       </c>
     </row>
     <row r="329">
-      <c r="A329">
+      <c r="A329" s="2">
         <f>IF(E329="","",COUNTA(E$2:E329))</f>
-        <v/>
       </c>
     </row>
     <row r="330">
-      <c r="A330">
+      <c r="A330" s="2">
         <f>IF(E330="","",COUNTA(E$2:E330))</f>
-        <v/>
       </c>
     </row>
     <row r="331">
-      <c r="A331">
+      <c r="A331" s="2">
         <f>IF(E331="","",COUNTA(E$2:E331))</f>
-        <v/>
       </c>
     </row>
     <row r="332">
-      <c r="A332">
+      <c r="A332" s="2">
         <f>IF(E332="","",COUNTA(E$2:E332))</f>
-        <v/>
       </c>
     </row>
     <row r="333">
-      <c r="A333">
+      <c r="A333" s="2">
         <f>IF(E333="","",COUNTA(E$2:E333))</f>
-        <v/>
       </c>
     </row>
     <row r="334">
-      <c r="A334">
+      <c r="A334" s="2">
         <f>IF(E334="","",COUNTA(E$2:E334))</f>
-        <v/>
       </c>
     </row>
     <row r="335">
-      <c r="A335">
+      <c r="A335" s="2">
         <f>IF(E335="","",COUNTA(E$2:E335))</f>
-        <v/>
       </c>
     </row>
     <row r="336">
-      <c r="A336">
+      <c r="A336" s="2">
         <f>IF(E336="","",COUNTA(E$2:E336))</f>
-        <v/>
       </c>
     </row>
     <row r="337">
-      <c r="A337">
+      <c r="A337" s="2">
         <f>IF(E337="","",COUNTA(E$2:E337))</f>
-        <v/>
       </c>
     </row>
     <row r="338">
-      <c r="A338">
+      <c r="A338" s="2">
         <f>IF(E338="","",COUNTA(E$2:E338))</f>
-        <v/>
       </c>
     </row>
     <row r="339">
-      <c r="A339">
+      <c r="A339" s="2">
         <f>IF(E339="","",COUNTA(E$2:E339))</f>
-        <v/>
       </c>
     </row>
     <row r="340">
-      <c r="A340">
+      <c r="A340" s="2">
         <f>IF(E340="","",COUNTA(E$2:E340))</f>
-        <v/>
       </c>
     </row>
     <row r="341">
-      <c r="A341">
+      <c r="A341" s="2">
         <f>IF(E341="","",COUNTA(E$2:E341))</f>
-        <v/>
       </c>
     </row>
     <row r="342">
-      <c r="A342">
+      <c r="A342" s="2">
         <f>IF(E342="","",COUNTA(E$2:E342))</f>
-        <v/>
       </c>
     </row>
     <row r="343">
-      <c r="A343">
+      <c r="A343" s="2">
         <f>IF(E343="","",COUNTA(E$2:E343))</f>
-        <v/>
       </c>
     </row>
     <row r="344">
-      <c r="A344">
+      <c r="A344" s="2">
         <f>IF(E344="","",COUNTA(E$2:E344))</f>
-        <v/>
       </c>
     </row>
     <row r="345">
-      <c r="A345">
+      <c r="A345" s="2">
         <f>IF(E345="","",COUNTA(E$2:E345))</f>
-        <v/>
       </c>
     </row>
     <row r="346">
-      <c r="A346">
+      <c r="A346" s="2">
         <f>IF(E346="","",COUNTA(E$2:E346))</f>
-        <v/>
       </c>
     </row>
     <row r="347">
-      <c r="A347">
+      <c r="A347" s="2">
         <f>IF(E347="","",COUNTA(E$2:E347))</f>
-        <v/>
       </c>
     </row>
     <row r="348">
-      <c r="A348">
+      <c r="A348" s="2">
         <f>IF(E348="","",COUNTA(E$2:E348))</f>
-        <v/>
       </c>
     </row>
     <row r="349">
-      <c r="A349">
+      <c r="A349" s="2">
         <f>IF(E349="","",COUNTA(E$2:E349))</f>
-        <v/>
       </c>
     </row>
     <row r="350">
-      <c r="A350">
+      <c r="A350" s="2">
         <f>IF(E350="","",COUNTA(E$2:E350))</f>
-        <v/>
       </c>
     </row>
     <row r="351">
-      <c r="A351">
+      <c r="A351" s="2">
         <f>IF(E351="","",COUNTA(E$2:E351))</f>
-        <v/>
       </c>
     </row>
     <row r="352">
-      <c r="A352">
+      <c r="A352" s="2">
         <f>IF(E352="","",COUNTA(E$2:E352))</f>
-        <v/>
       </c>
     </row>
     <row r="353">
-      <c r="A353">
+      <c r="A353" s="2">
         <f>IF(E353="","",COUNTA(E$2:E353))</f>
-        <v/>
       </c>
     </row>
     <row r="354">
-      <c r="A354">
+      <c r="A354" s="2">
         <f>IF(E354="","",COUNTA(E$2:E354))</f>
-        <v/>
       </c>
     </row>
     <row r="355">
-      <c r="A355">
+      <c r="A355" s="2">
         <f>IF(E355="","",COUNTA(E$2:E355))</f>
-        <v/>
       </c>
     </row>
     <row r="356">
-      <c r="A356">
+      <c r="A356" s="2">
         <f>IF(E356="","",COUNTA(E$2:E356))</f>
-        <v/>
       </c>
     </row>
     <row r="357">
-      <c r="A357">
+      <c r="A357" s="2">
         <f>IF(E357="","",COUNTA(E$2:E357))</f>
-        <v/>
       </c>
     </row>
     <row r="358">
-      <c r="A358">
+      <c r="A358" s="2">
         <f>IF(E358="","",COUNTA(E$2:E358))</f>
-        <v/>
       </c>
     </row>
     <row r="359">
-      <c r="A359">
+      <c r="A359" s="2">
         <f>IF(E359="","",COUNTA(E$2:E359))</f>
-        <v/>
       </c>
     </row>
     <row r="360">
-      <c r="A360">
+      <c r="A360" s="2">
         <f>IF(E360="","",COUNTA(E$2:E360))</f>
-        <v/>
       </c>
     </row>
     <row r="361">
-      <c r="A361">
+      <c r="A361" s="2">
         <f>IF(E361="","",COUNTA(E$2:E361))</f>
-        <v/>
       </c>
     </row>
     <row r="362">
-      <c r="A362">
+      <c r="A362" s="2">
         <f>IF(E362="","",COUNTA(E$2:E362))</f>
-        <v/>
       </c>
     </row>
     <row r="363">
-      <c r="A363">
+      <c r="A363" s="2">
         <f>IF(E363="","",COUNTA(E$2:E363))</f>
-        <v/>
       </c>
     </row>
     <row r="364">
-      <c r="A364">
+      <c r="A364" s="2">
         <f>IF(E364="","",COUNTA(E$2:E364))</f>
-        <v/>
       </c>
     </row>
     <row r="365">
-      <c r="A365">
+      <c r="A365" s="2">
         <f>IF(E365="","",COUNTA(E$2:E365))</f>
-        <v/>
       </c>
     </row>
     <row r="366">
-      <c r="A366">
+      <c r="A366" s="2">
         <f>IF(E366="","",COUNTA(E$2:E366))</f>
-        <v/>
       </c>
     </row>
     <row r="367">
-      <c r="A367">
+      <c r="A367" s="2">
         <f>IF(E367="","",COUNTA(E$2:E367))</f>
-        <v/>
       </c>
     </row>
     <row r="368">
-      <c r="A368">
+      <c r="A368" s="2">
         <f>IF(E368="","",COUNTA(E$2:E368))</f>
-        <v/>
       </c>
     </row>
     <row r="369">
-      <c r="A369">
+      <c r="A369" s="2">
         <f>IF(E369="","",COUNTA(E$2:E369))</f>
-        <v/>
       </c>
     </row>
     <row r="370">
-      <c r="A370">
+      <c r="A370" s="2">
         <f>IF(E370="","",COUNTA(E$2:E370))</f>
-        <v/>
       </c>
     </row>
     <row r="371">
-      <c r="A371">
+      <c r="A371" s="2">
         <f>IF(E371="","",COUNTA(E$2:E371))</f>
-        <v/>
       </c>
     </row>
     <row r="372">
-      <c r="A372">
+      <c r="A372" s="2">
         <f>IF(E372="","",COUNTA(E$2:E372))</f>
-        <v/>
       </c>
     </row>
     <row r="373">
-      <c r="A373">
+      <c r="A373" s="2">
         <f>IF(E373="","",COUNTA(E$2:E373))</f>
-        <v/>
       </c>
     </row>
     <row r="374">
-      <c r="A374">
+      <c r="A374" s="2">
         <f>IF(E374="","",COUNTA(E$2:E374))</f>
-        <v/>
       </c>
     </row>
     <row r="375">
-      <c r="A375">
+      <c r="A375" s="2">
         <f>IF(E375="","",COUNTA(E$2:E375))</f>
-        <v/>
       </c>
     </row>
     <row r="376">
-      <c r="A376">
+      <c r="A376" s="2">
         <f>IF(E376="","",COUNTA(E$2:E376))</f>
-        <v/>
       </c>
     </row>
     <row r="377">
-      <c r="A377">
+      <c r="A377" s="2">
         <f>IF(E377="","",COUNTA(E$2:E377))</f>
-        <v/>
       </c>
     </row>
     <row r="378">
-      <c r="A378">
+      <c r="A378" s="2">
         <f>IF(E378="","",COUNTA(E$2:E378))</f>
-        <v/>
       </c>
     </row>
     <row r="379">
-      <c r="A379">
+      <c r="A379" s="2">
         <f>IF(E379="","",COUNTA(E$2:E379))</f>
-        <v/>
       </c>
     </row>
     <row r="380">
-      <c r="A380">
+      <c r="A380" s="2">
         <f>IF(E380="","",COUNTA(E$2:E380))</f>
-        <v/>
       </c>
     </row>
     <row r="381">
-      <c r="A381">
+      <c r="A381" s="2">
         <f>IF(E381="","",COUNTA(E$2:E381))</f>
-        <v/>
       </c>
     </row>
     <row r="382">
-      <c r="A382">
+      <c r="A382" s="2">
         <f>IF(E382="","",COUNTA(E$2:E382))</f>
-        <v/>
       </c>
     </row>
     <row r="383">
-      <c r="A383">
+      <c r="A383" s="2">
         <f>IF(E383="","",COUNTA(E$2:E383))</f>
-        <v/>
       </c>
     </row>
     <row r="384">
-      <c r="A384">
+      <c r="A384" s="2">
         <f>IF(E384="","",COUNTA(E$2:E384))</f>
-        <v/>
       </c>
     </row>
     <row r="385">
-      <c r="A385">
+      <c r="A385" s="2">
         <f>IF(E385="","",COUNTA(E$2:E385))</f>
-        <v/>
       </c>
     </row>
     <row r="386">
-      <c r="A386">
+      <c r="A386" s="2">
         <f>IF(E386="","",COUNTA(E$2:E386))</f>
-        <v/>
       </c>
     </row>
     <row r="387">
-      <c r="A387">
+      <c r="A387" s="2">
         <f>IF(E387="","",COUNTA(E$2:E387))</f>
-        <v/>
       </c>
     </row>
     <row r="388">
-      <c r="A388">
+      <c r="A388" s="2">
         <f>IF(E388="","",COUNTA(E$2:E388))</f>
-        <v/>
       </c>
     </row>
     <row r="389">
-      <c r="A389">
+      <c r="A389" s="2">
         <f>IF(E389="","",COUNTA(E$2:E389))</f>
-        <v/>
       </c>
     </row>
     <row r="390">
-      <c r="A390">
+      <c r="A390" s="2">
         <f>IF(E390="","",COUNTA(E$2:E390))</f>
-        <v/>
       </c>
     </row>
     <row r="391">
-      <c r="A391">
+      <c r="A391" s="2">
         <f>IF(E391="","",COUNTA(E$2:E391))</f>
-        <v/>
       </c>
     </row>
     <row r="392">
-      <c r="A392">
+      <c r="A392" s="2">
         <f>IF(E392="","",COUNTA(E$2:E392))</f>
-        <v/>
       </c>
     </row>
     <row r="393">
-      <c r="A393">
+      <c r="A393" s="2">
         <f>IF(E393="","",COUNTA(E$2:E393))</f>
-        <v/>
       </c>
     </row>
     <row r="394">
-      <c r="A394">
+      <c r="A394" s="2">
         <f>IF(E394="","",COUNTA(E$2:E394))</f>
-        <v/>
       </c>
     </row>
     <row r="395">
-      <c r="A395">
+      <c r="A395" s="2">
         <f>IF(E395="","",COUNTA(E$2:E395))</f>
-        <v/>
       </c>
     </row>
     <row r="396">
-      <c r="A396">
+      <c r="A396" s="2">
         <f>IF(E396="","",COUNTA(E$2:E396))</f>
-        <v/>
       </c>
     </row>
     <row r="397">
-      <c r="A397">
+      <c r="A397" s="2">
         <f>IF(E397="","",COUNTA(E$2:E397))</f>
-        <v/>
       </c>
     </row>
     <row r="398">
-      <c r="A398">
+      <c r="A398" s="2">
         <f>IF(E398="","",COUNTA(E$2:E398))</f>
-        <v/>
       </c>
     </row>
     <row r="399">
-      <c r="A399">
+      <c r="A399" s="2">
         <f>IF(E399="","",COUNTA(E$2:E399))</f>
-        <v/>
       </c>
     </row>
     <row r="400">
-      <c r="A400">
+      <c r="A400" s="2">
         <f>IF(E400="","",COUNTA(E$2:E400))</f>
-        <v/>
       </c>
     </row>
     <row r="401">
-      <c r="A401">
+      <c r="A401" s="2">
         <f>IF(E401="","",COUNTA(E$2:E401))</f>
-        <v/>
       </c>
     </row>
     <row r="402">
-      <c r="A402">
+      <c r="A402" s="2">
         <f>IF(E402="","",COUNTA(E$2:E402))</f>
-        <v/>
       </c>
     </row>
     <row r="403">
-      <c r="A403">
+      <c r="A403" s="2">
         <f>IF(E403="","",COUNTA(E$2:E403))</f>
-        <v/>
       </c>
     </row>
     <row r="404">
-      <c r="A404">
+      <c r="A404" s="2">
         <f>IF(E404="","",COUNTA(E$2:E404))</f>
-        <v/>
       </c>
     </row>
     <row r="405">
-      <c r="A405">
+      <c r="A405" s="2">
         <f>IF(E405="","",COUNTA(E$2:E405))</f>
-        <v/>
       </c>
     </row>
     <row r="406">
-      <c r="A406">
+      <c r="A406" s="2">
         <f>IF(E406="","",COUNTA(E$2:E406))</f>
-        <v/>
       </c>
     </row>
     <row r="407">
-      <c r="A407">
+      <c r="A407" s="2">
         <f>IF(E407="","",COUNTA(E$2:E407))</f>
-        <v/>
       </c>
     </row>
     <row r="408">
-      <c r="A408">
+      <c r="A408" s="2">
         <f>IF(E408="","",COUNTA(E$2:E408))</f>
-        <v/>
       </c>
     </row>
     <row r="409">
-      <c r="A409">
+      <c r="A409" s="2">
         <f>IF(E409="","",COUNTA(E$2:E409))</f>
-        <v/>
       </c>
     </row>
     <row r="410">
-      <c r="A410">
+      <c r="A410" s="2">
         <f>IF(E410="","",COUNTA(E$2:E410))</f>
-        <v/>
       </c>
     </row>
     <row r="411">
-      <c r="A411">
+      <c r="A411" s="2">
         <f>IF(E411="","",COUNTA(E$2:E411))</f>
-        <v/>
       </c>
     </row>
     <row r="412">
-      <c r="A412">
+      <c r="A412" s="2">
         <f>IF(E412="","",COUNTA(E$2:E412))</f>
-        <v/>
       </c>
     </row>
     <row r="413">
-      <c r="A413">
+      <c r="A413" s="2">
         <f>IF(E413="","",COUNTA(E$2:E413))</f>
-        <v/>
       </c>
     </row>
     <row r="414">
-      <c r="A414">
+      <c r="A414" s="2">
         <f>IF(E414="","",COUNTA(E$2:E414))</f>
-        <v/>
       </c>
     </row>
     <row r="415">
-      <c r="A415">
+      <c r="A415" s="2">
         <f>IF(E415="","",COUNTA(E$2:E415))</f>
-        <v/>
       </c>
     </row>
     <row r="416">
-      <c r="A416">
+      <c r="A416" s="2">
         <f>IF(E416="","",COUNTA(E$2:E416))</f>
-        <v/>
       </c>
     </row>
     <row r="417">
-      <c r="A417">
+      <c r="A417" s="2">
         <f>IF(E417="","",COUNTA(E$2:E417))</f>
-        <v/>
       </c>
     </row>
     <row r="418">
-      <c r="A418">
+      <c r="A418" s="2">
         <f>IF(E418="","",COUNTA(E$2:E418))</f>
-        <v/>
       </c>
     </row>
     <row r="419">
-      <c r="A419">
+      <c r="A419" s="2">
         <f>IF(E419="","",COUNTA(E$2:E419))</f>
-        <v/>
       </c>
     </row>
     <row r="420">
-      <c r="A420">
+      <c r="A420" s="2">
         <f>IF(E420="","",COUNTA(E$2:E420))</f>
-        <v/>
       </c>
     </row>
     <row r="421">
-      <c r="A421">
+      <c r="A421" s="2">
         <f>IF(E421="","",COUNTA(E$2:E421))</f>
-        <v/>
       </c>
     </row>
     <row r="422">
-      <c r="A422">
+      <c r="A422" s="2">
         <f>IF(E422="","",COUNTA(E$2:E422))</f>
-        <v/>
       </c>
     </row>
     <row r="423">
-      <c r="A423">
+      <c r="A423" s="2">
         <f>IF(E423="","",COUNTA(E$2:E423))</f>
-        <v/>
       </c>
     </row>
     <row r="424">
-      <c r="A424">
+      <c r="A424" s="2">
         <f>IF(E424="","",COUNTA(E$2:E424))</f>
-        <v/>
       </c>
     </row>
     <row r="425">
-      <c r="A425">
+      <c r="A425" s="2">
         <f>IF(E425="","",COUNTA(E$2:E425))</f>
-        <v/>
       </c>
     </row>
     <row r="426">
-      <c r="A426">
+      <c r="A426" s="2">
         <f>IF(E426="","",COUNTA(E$2:E426))</f>
-        <v/>
       </c>
     </row>
     <row r="427">
-      <c r="A427">
+      <c r="A427" s="2">
         <f>IF(E427="","",COUNTA(E$2:E427))</f>
-        <v/>
       </c>
     </row>
     <row r="428">
-      <c r="A428">
+      <c r="A428" s="2">
         <f>IF(E428="","",COUNTA(E$2:E428))</f>
-        <v/>
       </c>
     </row>
     <row r="429">
-      <c r="A429">
+      <c r="A429" s="2">
         <f>IF(E429="","",COUNTA(E$2:E429))</f>
-        <v/>
       </c>
     </row>
     <row r="430">
-      <c r="A430">
+      <c r="A430" s="2">
         <f>IF(E430="","",COUNTA(E$2:E430))</f>
-        <v/>
       </c>
     </row>
     <row r="431">
-      <c r="A431">
+      <c r="A431" s="2">
         <f>IF(E431="","",COUNTA(E$2:E431))</f>
-        <v/>
       </c>
     </row>
     <row r="432">
-      <c r="A432">
+      <c r="A432" s="2">
         <f>IF(E432="","",COUNTA(E$2:E432))</f>
-        <v/>
       </c>
     </row>
     <row r="433">
-      <c r="A433">
+      <c r="A433" s="2">
         <f>IF(E433="","",COUNTA(E$2:E433))</f>
-        <v/>
       </c>
     </row>
     <row r="434">
-      <c r="A434">
+      <c r="A434" s="2">
         <f>IF(E434="","",COUNTA(E$2:E434))</f>
-        <v/>
       </c>
     </row>
     <row r="435">
-      <c r="A435">
+      <c r="A435" s="2">
         <f>IF(E435="","",COUNTA(E$2:E435))</f>
-        <v/>
       </c>
     </row>
     <row r="436">
-      <c r="A436">
+      <c r="A436" s="2">
         <f>IF(E436="","",COUNTA(E$2:E436))</f>
-        <v/>
       </c>
     </row>
     <row r="437">
-      <c r="A437">
+      <c r="A437" s="2">
         <f>IF(E437="","",COUNTA(E$2:E437))</f>
-        <v/>
       </c>
     </row>
     <row r="438">
-      <c r="A438">
+      <c r="A438" s="2">
         <f>IF(E438="","",COUNTA(E$2:E438))</f>
-        <v/>
       </c>
     </row>
     <row r="439">
-      <c r="A439">
+      <c r="A439" s="2">
         <f>IF(E439="","",COUNTA(E$2:E439))</f>
-        <v/>
       </c>
     </row>
     <row r="440">
-      <c r="A440">
+      <c r="A440" s="2">
         <f>IF(E440="","",COUNTA(E$2:E440))</f>
-        <v/>
       </c>
     </row>
     <row r="441">
-      <c r="A441">
+      <c r="A441" s="2">
         <f>IF(E441="","",COUNTA(E$2:E441))</f>
-        <v/>
       </c>
     </row>
     <row r="442">
-      <c r="A442">
+      <c r="A442" s="2">
         <f>IF(E442="","",COUNTA(E$2:E442))</f>
-        <v/>
       </c>
     </row>
     <row r="443">
-      <c r="A443">
+      <c r="A443" s="2">
         <f>IF(E443="","",COUNTA(E$2:E443))</f>
-        <v/>
       </c>
     </row>
     <row r="444">
-      <c r="A444">
+      <c r="A444" s="2">
         <f>IF(E444="","",COUNTA(E$2:E444))</f>
-        <v/>
       </c>
     </row>
     <row r="445">
-      <c r="A445">
+      <c r="A445" s="2">
         <f>IF(E445="","",COUNTA(E$2:E445))</f>
-        <v/>
       </c>
     </row>
     <row r="446">
-      <c r="A446">
+      <c r="A446" s="2">
         <f>IF(E446="","",COUNTA(E$2:E446))</f>
-        <v/>
       </c>
     </row>
     <row r="447">
-      <c r="A447">
+      <c r="A447" s="2">
         <f>IF(E447="","",COUNTA(E$2:E447))</f>
-        <v/>
       </c>
     </row>
     <row r="448">
-      <c r="A448">
+      <c r="A448" s="2">
         <f>IF(E448="","",COUNTA(E$2:E448))</f>
-        <v/>
       </c>
     </row>
     <row r="449">
-      <c r="A449">
+      <c r="A449" s="2">
         <f>IF(E449="","",COUNTA(E$2:E449))</f>
-        <v/>
       </c>
     </row>
     <row r="450">
-      <c r="A450">
+      <c r="A450" s="2">
         <f>IF(E450="","",COUNTA(E$2:E450))</f>
-        <v/>
       </c>
     </row>
     <row r="451">
-      <c r="A451">
+      <c r="A451" s="2">
         <f>IF(E451="","",COUNTA(E$2:E451))</f>
-        <v/>
       </c>
     </row>
     <row r="452">
-      <c r="A452">
+      <c r="A452" s="2">
         <f>IF(E452="","",COUNTA(E$2:E452))</f>
-        <v/>
       </c>
     </row>
     <row r="453">
-      <c r="A453">
+      <c r="A453" s="2">
         <f>IF(E453="","",COUNTA(E$2:E453))</f>
-        <v/>
       </c>
     </row>
     <row r="454">
-      <c r="A454">
+      <c r="A454" s="2">
         <f>IF(E454="","",COUNTA(E$2:E454))</f>
-        <v/>
       </c>
     </row>
     <row r="455">
-      <c r="A455">
+      <c r="A455" s="2">
         <f>IF(E455="","",COUNTA(E$2:E455))</f>
-        <v/>
       </c>
     </row>
     <row r="456">
-      <c r="A456">
+      <c r="A456" s="2">
         <f>IF(E456="","",COUNTA(E$2:E456))</f>
-        <v/>
       </c>
     </row>
     <row r="457">
-      <c r="A457">
+      <c r="A457" s="2">
         <f>IF(E457="","",COUNTA(E$2:E457))</f>
-        <v/>
       </c>
     </row>
     <row r="458">
-      <c r="A458">
+      <c r="A458" s="2">
         <f>IF(E458="","",COUNTA(E$2:E458))</f>
-        <v/>
       </c>
     </row>
     <row r="459">
-      <c r="A459">
+      <c r="A459" s="2">
         <f>IF(E459="","",COUNTA(E$2:E459))</f>
-        <v/>
       </c>
     </row>
     <row r="460">
-      <c r="A460">
+      <c r="A460" s="2">
         <f>IF(E460="","",COUNTA(E$2:E460))</f>
-        <v/>
       </c>
     </row>
     <row r="461">
-      <c r="A461">
+      <c r="A461" s="2">
         <f>IF(E461="","",COUNTA(E$2:E461))</f>
-        <v/>
       </c>
     </row>
     <row r="462">
-      <c r="A462">
+      <c r="A462" s="2">
         <f>IF(E462="","",COUNTA(E$2:E462))</f>
-        <v/>
       </c>
     </row>
     <row r="463">
-      <c r="A463">
+      <c r="A463" s="2">
         <f>IF(E463="","",COUNTA(E$2:E463))</f>
-        <v/>
       </c>
     </row>
     <row r="464">
-      <c r="A464">
+      <c r="A464" s="2">
         <f>IF(E464="","",COUNTA(E$2:E464))</f>
-        <v/>
       </c>
     </row>
     <row r="465">
-      <c r="A465">
+      <c r="A465" s="2">
         <f>IF(E465="","",COUNTA(E$2:E465))</f>
-        <v/>
       </c>
     </row>
     <row r="466">
-      <c r="A466">
+      <c r="A466" s="2">
         <f>IF(E466="","",COUNTA(E$2:E466))</f>
-        <v/>
       </c>
     </row>
     <row r="467">
-      <c r="A467">
+      <c r="A467" s="2">
         <f>IF(E467="","",COUNTA(E$2:E467))</f>
-        <v/>
       </c>
     </row>
     <row r="468">
-      <c r="A468">
+      <c r="A468" s="2">
         <f>IF(E468="","",COUNTA(E$2:E468))</f>
-        <v/>
       </c>
     </row>
     <row r="469">
-      <c r="A469">
+      <c r="A469" s="2">
         <f>IF(E469="","",COUNTA(E$2:E469))</f>
-        <v/>
       </c>
     </row>
     <row r="470">
-      <c r="A470">
+      <c r="A470" s="2">
         <f>IF(E470="","",COUNTA(E$2:E470))</f>
-        <v/>
       </c>
     </row>
     <row r="471">
-      <c r="A471">
+      <c r="A471" s="2">
         <f>IF(E471="","",COUNTA(E$2:E471))</f>
-        <v/>
       </c>
     </row>
     <row r="472">
-      <c r="A472">
+      <c r="A472" s="2">
         <f>IF(E472="","",COUNTA(E$2:E472))</f>
-        <v/>
       </c>
     </row>
     <row r="473">
-      <c r="A473">
+      <c r="A473" s="2">
         <f>IF(E473="","",COUNTA(E$2:E473))</f>
-        <v/>
       </c>
     </row>
     <row r="474">
-      <c r="A474">
+      <c r="A474" s="2">
         <f>IF(E474="","",COUNTA(E$2:E474))</f>
-        <v/>
       </c>
     </row>
     <row r="475">
-      <c r="A475">
+      <c r="A475" s="2">
         <f>IF(E475="","",COUNTA(E$2:E475))</f>
-        <v/>
       </c>
     </row>
     <row r="476">
-      <c r="A476">
+      <c r="A476" s="2">
         <f>IF(E476="","",COUNTA(E$2:E476))</f>
-        <v/>
       </c>
     </row>
     <row r="477">
-      <c r="A477">
+      <c r="A477" s="2">
         <f>IF(E477="","",COUNTA(E$2:E477))</f>
-        <v/>
       </c>
     </row>
     <row r="478">
-      <c r="A478">
+      <c r="A478" s="2">
         <f>IF(E478="","",COUNTA(E$2:E478))</f>
-        <v/>
       </c>
     </row>
     <row r="479">
-      <c r="A479">
+      <c r="A479" s="2">
         <f>IF(E479="","",COUNTA(E$2:E479))</f>
-        <v/>
       </c>
     </row>
     <row r="480">
-      <c r="A480">
+      <c r="A480" s="2">
         <f>IF(E480="","",COUNTA(E$2:E480))</f>
-        <v/>
       </c>
     </row>
     <row r="481">
-      <c r="A481">
+      <c r="A481" s="2">
         <f>IF(E481="","",COUNTA(E$2:E481))</f>
-        <v/>
       </c>
     </row>
     <row r="482">
-      <c r="A482">
+      <c r="A482" s="2">
         <f>IF(E482="","",COUNTA(E$2:E482))</f>
-        <v/>
       </c>
     </row>
     <row r="483">
-      <c r="A483">
+      <c r="A483" s="2">
         <f>IF(E483="","",COUNTA(E$2:E483))</f>
-        <v/>
       </c>
     </row>
     <row r="484">
-      <c r="A484">
+      <c r="A484" s="2">
         <f>IF(E484="","",COUNTA(E$2:E484))</f>
-        <v/>
       </c>
     </row>
     <row r="485">
-      <c r="A485">
+      <c r="A485" s="2">
         <f>IF(E485="","",COUNTA(E$2:E485))</f>
-        <v/>
       </c>
     </row>
     <row r="486">
-      <c r="A486">
+      <c r="A486" s="2">
         <f>IF(E486="","",COUNTA(E$2:E486))</f>
-        <v/>
       </c>
     </row>
     <row r="487">
-      <c r="A487">
+      <c r="A487" s="2">
         <f>IF(E487="","",COUNTA(E$2:E487))</f>
-        <v/>
       </c>
     </row>
     <row r="488">
-      <c r="A488">
+      <c r="A488" s="2">
         <f>IF(E488="","",COUNTA(E$2:E488))</f>
-        <v/>
       </c>
     </row>
     <row r="489">
-      <c r="A489">
+      <c r="A489" s="2">
         <f>IF(E489="","",COUNTA(E$2:E489))</f>
-        <v/>
       </c>
     </row>
     <row r="490">
-      <c r="A490">
+      <c r="A490" s="2">
         <f>IF(E490="","",COUNTA(E$2:E490))</f>
-        <v/>
       </c>
     </row>
     <row r="491">
-      <c r="A491">
+      <c r="A491" s="2">
         <f>IF(E491="","",COUNTA(E$2:E491))</f>
-        <v/>
       </c>
     </row>
     <row r="492">
-      <c r="A492">
+      <c r="A492" s="2">
         <f>IF(E492="","",COUNTA(E$2:E492))</f>
-        <v/>
       </c>
     </row>
     <row r="493">
-      <c r="A493">
+      <c r="A493" s="2">
         <f>IF(E493="","",COUNTA(E$2:E493))</f>
-        <v/>
       </c>
     </row>
     <row r="494">
-      <c r="A494">
+      <c r="A494" s="2">
         <f>IF(E494="","",COUNTA(E$2:E494))</f>
-        <v/>
       </c>
     </row>
     <row r="495">
-      <c r="A495">
+      <c r="A495" s="2">
         <f>IF(E495="","",COUNTA(E$2:E495))</f>
-        <v/>
       </c>
     </row>
     <row r="496">
-      <c r="A496">
+      <c r="A496" s="2">
         <f>IF(E496="","",COUNTA(E$2:E496))</f>
-        <v/>
       </c>
     </row>
     <row r="497">
-      <c r="A497">
+      <c r="A497" s="2">
         <f>IF(E497="","",COUNTA(E$2:E497))</f>
-        <v/>
       </c>
     </row>
     <row r="498">
-      <c r="A498">
+      <c r="A498" s="2">
         <f>IF(E498="","",COUNTA(E$2:E498))</f>
-        <v/>
       </c>
     </row>
     <row r="499">
-      <c r="A499">
+      <c r="A499" s="2">
         <f>IF(E499="","",COUNTA(E$2:E499))</f>
-        <v/>
       </c>
     </row>
     <row r="500">
-      <c r="A500">
+      <c r="A500" s="2">
         <f>IF(E500="","",COUNTA(E$2:E500))</f>
-        <v/>
       </c>
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid" error="Pick one from the dropdown." type="list">
+    <dataValidation type="list" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" sqref="E2:E500">
       <formula1>"Amazon,Flipkart,Meesho,Firstcry,Myntra"</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid" error="Pick one from the dropdown." type="list">
+    <dataValidation type="list" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" sqref="H2:H500">
       <formula1>"Y,N"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid" error="Pick one from the dropdown." type="list">
+    <dataValidation type="list" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" sqref="I2:I500">
       <formula1>"Combo,Single,Qwantity,MOQ"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Master SKU sample: page column order A-T, X-AG, AI-AK (33 cols), Floor Margin header
</commit_message>
<xml_diff>
--- a/skuwisedata/master_sku_sample.xlsx
+++ b/skuwisedata/master_sku_sample.xlsx
@@ -86,7 +86,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AE500"/>
+  <dimension ref="A1:AG500"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -94,32 +94,34 @@
     <col min="3" max="3" width="14" customWidth="1"/>
     <col min="4" max="4" width="18" customWidth="1"/>
     <col min="5" max="5" width="11" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="12" customWidth="1"/>
-    <col min="8" max="8" width="13" customWidth="1"/>
-    <col min="9" max="9" width="11" customWidth="1"/>
-    <col min="10" max="10" width="14" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="12" customWidth="1"/>
+    <col min="9" max="9" width="14" customWidth="1"/>
+    <col min="10" max="10" width="11" customWidth="1"/>
     <col min="11" max="11" width="14" customWidth="1"/>
-    <col min="12" max="12" width="22" customWidth="1"/>
-    <col min="13" max="13" width="10" customWidth="1"/>
-    <col min="14" max="14" width="14" customWidth="1"/>
-    <col min="15" max="15" width="18" customWidth="1"/>
-    <col min="16" max="16" width="20" customWidth="1"/>
-    <col min="17" max="17" width="20" customWidth="1"/>
-    <col min="18" max="18" width="10" customWidth="1"/>
-    <col min="19" max="19" width="10" customWidth="1"/>
-    <col min="20" max="20" width="8" customWidth="1"/>
+    <col min="12" max="12" width="14" customWidth="1"/>
+    <col min="13" max="13" width="22" customWidth="1"/>
+    <col min="14" max="14" width="10" customWidth="1"/>
+    <col min="15" max="15" width="9" customWidth="1"/>
+    <col min="16" max="16" width="7" customWidth="1"/>
+    <col min="17" max="17" width="14" customWidth="1"/>
+    <col min="18" max="18" width="18" customWidth="1"/>
+    <col min="19" max="19" width="20" customWidth="1"/>
+    <col min="20" max="20" width="20" customWidth="1"/>
     <col min="21" max="21" width="10" customWidth="1"/>
-    <col min="22" max="22" width="14" customWidth="1"/>
-    <col min="23" max="23" width="14" customWidth="1"/>
-    <col min="24" max="24" width="14" customWidth="1"/>
-    <col min="25" max="25" width="14" customWidth="1"/>
-    <col min="26" max="26" width="18" customWidth="1"/>
+    <col min="22" max="22" width="10" customWidth="1"/>
+    <col min="23" max="23" width="8" customWidth="1"/>
+    <col min="24" max="24" width="10" customWidth="1"/>
+    <col min="25" max="25" width="11" customWidth="1"/>
+    <col min="26" max="26" width="14" customWidth="1"/>
     <col min="27" max="27" width="14" customWidth="1"/>
-    <col min="28" max="28" width="12" customWidth="1"/>
-    <col min="29" max="29" width="11" customWidth="1"/>
+    <col min="28" max="28" width="14" customWidth="1"/>
+    <col min="29" max="29" width="14" customWidth="1"/>
     <col min="30" max="30" width="18" customWidth="1"/>
-    <col min="31" max="31" width="13" customWidth="1"/>
+    <col min="31" max="31" width="14" customWidth="1"/>
+    <col min="32" max="32" width="12" customWidth="1"/>
+    <col min="33" max="33" width="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -150,130 +152,140 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Platform Seller</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Brand</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Vertical</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Non Returnable</t>
-        </is>
-      </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>Return Type</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Sub Category</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Color</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Mapped</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>MOQ</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>ASIN</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Other Listing Id</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>SKU</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Master Sku</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>COP</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>HSN</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Tax %</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Packaging</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>Margin</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Final COP</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Floor Margin</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Auto Margin</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Auto %</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Manual Margin</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Manual Settlement</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Amazon Add Rs</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Max Step %</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>Final COP</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>Expected Settlement</t>
-        </is>
-      </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Selling Price</t>
         </is>
@@ -2775,14 +2787,11 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="3">
+  <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" sqref="E2:E500">
       <formula1>"Amazon,Flipkart,Meesho,Firstcry,Myntra"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" sqref="H2:H500">
-      <formula1>"Y,N"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" sqref="I2:I500">
+    <dataValidation type="list" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" sqref="J2:J500">
       <formula1>"Combo,Single,Qwantity,MOQ"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>